<commit_message>
content: add Introduction sheet to both Excel workbooks
</commit_message>
<xml_diff>
--- a/Verbes Transitifs.xlsx
+++ b/Verbes Transitifs.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Transitifs Directs (COD)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transitifs Indirects (COI)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Introduction" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transitifs Directs (COD)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Transitifs Indirects (COI)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,338 +415,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Sujet</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Options</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>FeedbackCorrect</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>FeedbackIncorrect</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MultipleChoice</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Lequel de ces verbes est un verbe transitif direct (qui prend un COD sans préposition) ?</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>manger, parler, ressembler, sourire</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>manger</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Correct ! On dit 'manger quelque chose'.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Faux. 'Manger' prend un objet direct (ex: manger une pomme).</t>
+          <t>Les Verbes Transitifs en Français</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FillInBlank</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Nous ___ la télévision tous les soirs.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>regardons</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Très bien ! 'Regarder' est un verbe transitif direct.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Incorrect. Le verbe est 'regarder' conjugué avec 'nous'.</t>
+          <t>Qu'est-ce qu'un verbe transitif ?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TrueFalse</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Un verbe transitif direct est suivi immédiatement de son objet, sans préposition comme 'à' ou 'de'.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Vrai</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>C'est exact ! Ex: Je lis un livre.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>C'est faux, c'est justement la définition du transitif direct.</t>
+          <t>Un verbe transitif est un verbe qui a besoin d'un complément d'objet pour compléter son sens.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OddOneOut</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Trouvez le verbe qui N'EST PAS transitif direct :</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>acheter, vendre, répondre, donner</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>répondre</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Correct ! On 'répond À quelqu'un' (transitif indirect).</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Incorrect. 'Répondre' construit avec la préposition 'à'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MultipleChoice</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Dans la phrase 'Elle lit ce poème', quelle est la fonction de 'ce poème' ?</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>COD, COI, Sujet</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Bravo ! C'est le Complément d'Objet Direct du verbe 'lit'.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Faux, c'est l'objet direct car il n'y a pas de préposition.</t>
+          <t>On distingue deux catégories : les verbes transitifs DIRECTS et les verbes transitifs INDIRECTS.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FillInBlank</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ils ont ___ leur maison l'année dernière.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>vendu</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Correct ! Vendre (quelque chose).</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Incorrect. 'ont vendu' est transitif direct.</t>
+          <t>Exemple</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MultipleChoice</t>
+          <t>Transitif Direct (COD)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Quel pronom remplace le COD dans : 'Je mange la pomme' ?</t>
+          <t>Le verbe se construit SANS préposition avant son complément.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Je lui mange, Je la mange, Je y mange</t>
+          <t>Verbe + complément direct</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Je la mange</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Parfait ! 'la' remplace 'la pomme'.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Faux, c'est 'la'.</t>
+          <t>Je mange une pomme. / Il lit un livre.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TrueFalse</t>
+          <t>Transitif Indirect (COI)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Le participe passé conjugué avec 'avoir' s'accorde avec le COD s'il est placé APRÈS le verbe.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Le verbe se construit AVEC une préposition (à, de) avant son complément.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Verbe + à/de + complément</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Faux</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Exact, il s'accorde seulement s'il est mis AVANT le verbe !</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Attention ! Il s'accorde uniquement si le COD le précède avant le verbe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MultipleChoice</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Choisis la bonne phrase :</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>J'écoute à la radio, J'écoute la radio, J'écoute de la radio</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>J'écoute la radio</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Bravo ! Écouter est transitif direct en français.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>En français, 'écouter' ne prend pas de préposition.</t>
+          <t>Je parle à Marc. / Il se souvient de toi.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FillInBlank</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Tu ___ ton temps avec ces bêtises.</t>
-        </is>
-      </c>
+          <t>Pronoms de remplacement</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>perds</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Correct, 'perdre' est transitif direct.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>C'est le verbe 'perdre'.</t>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pour le COD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Utiliser : le, la, l', les</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Je mange la pomme → Je la mange.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Pour le COI avec 'à' (personne)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Utiliser : lui, leur</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Je parle à Marc → Je lui parle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pour le COI avec 'à' (chose)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Utiliser : y</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Je pense à ce projet → J'y pense.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pour le COI avec 'de'</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Utiliser : en</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Il parle de son voyage → Il en parle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Conseil</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Posez la question 'Qui ?' ou 'Quoi ?' directement après le verbe → COD (sans préposition). Si vous avez besoin de 'à qui ?' ou 'de quoi ?' → COI (avec préposition).</t>
         </is>
       </c>
     </row>
@@ -803,27 +671,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lequel de ces verbes est transitif indirect (se construit avec une préposition 'à' ou 'de') ?</t>
+          <t>Lequel de ces verbes est un verbe transitif direct (qui prend un COD sans préposition) ?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>parler, voir, écouter</t>
+          <t>manger, parler, ressembler, sourire</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>parler</t>
+          <t>manger</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Correct ! On 'parle À quelqu'un' ou 'DE quelque chose'.</t>
+          <t>Correct ! On dit 'manger quelque chose'.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Faux. Voir et écouter sont directs. Parler nécessite une préposition.</t>
+          <t>Faux. 'Manger' prend un objet direct (ex: manger une pomme).</t>
         </is>
       </c>
     </row>
@@ -835,23 +703,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Je téléphone ___ mon frère.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Nous ___ la télévision tous les soirs.</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>à</t>
+          <t>regardons</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Très bien ! Téléphoner À quelqu'un.</t>
+          <t>Très bien ! 'Regarder' est un verbe transitif direct.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Il manque la préposition 'à'.</t>
+          <t>Incorrect. Le verbe est 'regarder' conjugué avec 'nous'.</t>
         </is>
       </c>
     </row>
@@ -863,10 +730,9 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Un verbe transitif indirect a besoin d'une préposition pour introduire son objet.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Un verbe transitif direct est suivi immédiatement de son objet, sans préposition comme 'à' ou 'de'.</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Vrai</t>
@@ -874,12 +740,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>C'est exact, contrairement aux verbes transitifs directs.</t>
+          <t>C'est exact ! Ex: Je lis un livre.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>C'est faux, la préposition est obligatoire.</t>
+          <t>C'est faux, c'est justement la définition du transitif direct.</t>
         </is>
       </c>
     </row>
@@ -891,27 +757,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Choisissez le verbe qui N'EST PAS transitif indirect avec 'à' :</t>
+          <t>Trouvez le verbe qui N'EST PAS transitif direct :</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ressembler à, penser à, oublier, plaire à</t>
+          <t>acheter, vendre, répondre, donner</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>oublier</t>
+          <t>répondre</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Correct ! 'Oublier' est transitif direct (oublier quelque chose/quelqu'un).</t>
+          <t>Correct ! On 'répond À quelqu'un' (transitif indirect).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Incorrect. Oublier est direct.</t>
+          <t>Incorrect. 'Répondre' construit avec la préposition 'à'.</t>
         </is>
       </c>
     </row>
@@ -923,27 +789,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quel pronom remplace le COI dans : 'Je parle à Marie' ?</t>
+          <t>Dans la phrase 'Elle lit ce poème', quelle est la fonction de 'ce poème' ?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Je la parle, Je lui parle, Je le parle</t>
+          <t>COD, COI, Sujet</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Je lui parle</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bravo ! 'lui' remplace un nom de personne introduit par 'à'.</t>
+          <t>Bravo ! C'est le Complément d'Objet Direct du verbe 'lit'.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Faux, c'est 'lui'.</t>
+          <t>Faux, c'est l'objet direct car il n'y a pas de préposition.</t>
         </is>
       </c>
     </row>
@@ -955,23 +821,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Il se souvient ___ cet événement.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Ils ont ___ leur maison l'année dernière.</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>vendu</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Correct ! Se souvenir DE quelque chose.</t>
+          <t>Correct ! Vendre (quelque chose).</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Se souvenir prend toujours la préposition 'de'.</t>
+          <t>Incorrect. 'ont vendu' est transitif direct.</t>
         </is>
       </c>
     </row>
@@ -983,27 +848,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Quel pronom remplace le COI introduit par 'de' : 'Il parle de son voyage' ?</t>
+          <t>Quel pronom remplace le COD dans : 'Je mange la pomme' ?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Il lui parle, Il en parle, Il y parle</t>
+          <t>Je lui mange, Je la mange, Je y mange</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Il en parle</t>
+          <t>Je la mange</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Parfait ! 'en' remplace un groupe nominal introduit par 'de'.</t>
+          <t>Parfait ! 'la' remplace 'la pomme'.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Faux, c'est 'en'.</t>
+          <t>Faux, c'est 'la'.</t>
         </is>
       </c>
     </row>
@@ -1015,10 +880,9 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>On peut utiliser le pronom 'lui' pour remplacer des objets inanimés introduits par 'à'.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Le participe passé conjugué avec 'avoir' s'accorde avec le COD s'il est placé APRÈS le verbe.</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Faux</t>
@@ -1026,12 +890,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Exact ! Pour les objets inanimés on utilise 'y' (Je pense à la maison -&gt; j'y pense).</t>
+          <t>Exact, il s'accorde seulement s'il est mis AVANT le verbe !</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Faux. On utilise 'y' pour les objets, 'lui' est pour les personnes isolées.</t>
+          <t>Attention ! Il s'accorde uniquement si le COD le précède avant le verbe.</t>
         </is>
       </c>
     </row>
@@ -1048,22 +912,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Je joue le piano, Je joue du piano</t>
+          <t>J'écoute à la radio, J'écoute la radio, J'écoute de la radio</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Je joue du piano</t>
+          <t>J'écoute la radio</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bravo ! Jouer d'un instrument = COI avec 'de'.</t>
+          <t>Bravo ! Écouter est transitif direct en français.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Faux. Jouer d'un instrument prend 'de'.</t>
+          <t>En français, 'écouter' ne prend pas de préposition.</t>
         </is>
       </c>
     </row>
@@ -1075,10 +939,350 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Tu ___ ton temps avec ces bêtises.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>perds</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Correct, 'perdre' est transitif direct.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>C'est le verbe 'perdre'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>FeedbackCorrect</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>FeedbackIncorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MultipleChoice</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Lequel de ces verbes est transitif indirect (se construit avec une préposition 'à' ou 'de') ?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>parler, voir, écouter</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Correct ! On 'parle À quelqu'un' ou 'DE quelque chose'.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Faux. Voir et écouter sont directs. Parler nécessite une préposition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FillInBlank</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Je téléphone ___ mon frère.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>à</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Très bien ! Téléphoner À quelqu'un.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Il manque la préposition 'à'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TrueFalse</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Un verbe transitif indirect a besoin d'une préposition pour introduire son objet.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Vrai</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>C'est exact, contrairement aux verbes transitifs directs.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>C'est faux, la préposition est obligatoire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OddOneOut</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Choisissez le verbe qui N'EST PAS transitif indirect avec 'à' :</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ressembler à, penser à, oublier, plaire à</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>oublier</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Correct ! 'Oublier' est transitif direct (oublier quelque chose/quelqu'un).</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Incorrect. Oublier est direct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MultipleChoice</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Quel pronom remplace le COI dans : 'Je parle à Marie' ?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Je la parle, Je lui parle, Je le parle</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Je lui parle</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bravo ! 'lui' remplace un nom de personne introduit par 'à'.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Faux, c'est 'lui'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FillInBlank</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Il se souvient ___ cet événement.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Correct ! Se souvenir DE quelque chose.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Se souvenir prend toujours la préposition 'de'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MultipleChoice</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Quel pronom remplace le COI introduit par 'de' : 'Il parle de son voyage' ?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Il lui parle, Il en parle, Il y parle</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Il en parle</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Parfait ! 'en' remplace un groupe nominal introduit par 'de'.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Faux, c'est 'en'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TrueFalse</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>On peut utiliser le pronom 'lui' pour remplacer des objets inanimés introduits par 'à'.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Faux</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Exact ! Pour les objets inanimés on utilise 'y' (Je pense à la maison -&gt; j'y pense).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Faux. On utilise 'y' pour les objets, 'lui' est pour les personnes isolées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MultipleChoice</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Choisis la bonne phrase :</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Je joue le piano, Je joue du piano</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Je joue du piano</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bravo ! Jouer d'un instrument = COI avec 'de'.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Faux. Jouer d'un instrument prend 'de'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FillInBlank</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Nous nous intéressons ___ ce projet.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>à</t>

</xml_diff>